<commit_message>
still working on test 1 plus
</commit_message>
<xml_diff>
--- a/prosp_draft_data.xlsx
+++ b/prosp_draft_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kristina/Documents/GitHub/phd/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358FAC01-BA95-B94F-9CA4-3A435E255B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D589B06-2792-AF4D-BDA3-AC4F64C6BBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="32120" windowHeight="19120" xr2:uid="{C3B414E7-4F74-B640-BD11-B6FEEAE78456}"/>
+    <workbookView xWindow="-4680" yWindow="-20680" windowWidth="32120" windowHeight="19020" xr2:uid="{C3B414E7-4F74-B640-BD11-B6FEEAE78456}"/>
   </bookViews>
   <sheets>
     <sheet name="drafting database" sheetId="2" r:id="rId1"/>
@@ -2799,7 +2799,7 @@
         <v>68</v>
       </c>
       <c r="B35" s="2">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>218</v>

</xml_diff>